<commit_message>
creat test data vovantuananh
</commit_message>
<xml_diff>
--- a/java22 database design/Java22 TuanAnh Database Design.xlsx
+++ b/java22 database design/Java22 TuanAnh Database Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LearningJava++\Java22\3.Database\java22 database design\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D0BD0A-8B3E-493E-8CB9-C6D9651683FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A29C3C-F42B-4A15-AAAC-893A115DD33A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="937" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="937" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="B1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -881,7 +881,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="543">
   <si>
     <t>NhanVien</t>
   </si>
@@ -2172,15 +2172,6 @@
     <t>C03_SALES_PRICE</t>
   </si>
   <si>
-    <t>C00_SUPPLIER_ID</t>
-  </si>
-  <si>
-    <t>C00_SUPPLIER_NAME</t>
-  </si>
-  <si>
-    <t>C00_SUPPLIER_TAX</t>
-  </si>
-  <si>
     <t>T100_SUPPLIER</t>
   </si>
   <si>
@@ -2527,6 +2518,9 @@
   </si>
   <si>
     <t>C13_EMPLOYEE_PASSWORD</t>
+  </si>
+  <si>
+    <t>C101_BUY_PRICE</t>
   </si>
 </sst>
 </file>
@@ -2996,6 +2990,16 @@
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3009,25 +3013,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5733,16 +5727,16 @@
     </row>
     <row r="72" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="73" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C73" s="65" t="s">
+      <c r="C73" s="70" t="s">
         <v>277</v>
       </c>
-      <c r="D73" s="65"/>
-      <c r="E73" s="65"/>
+      <c r="D73" s="70"/>
+      <c r="E73" s="70"/>
     </row>
     <row r="74" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C74" s="65"/>
-      <c r="D74" s="65"/>
-      <c r="E74" s="65"/>
+      <c r="C74" s="70"/>
+      <c r="D74" s="70"/>
+      <c r="E74" s="70"/>
     </row>
     <row r="75" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="76" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5766,14 +5760,14 @@
     </row>
     <row r="78" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="79" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C79" s="65" t="s">
+      <c r="C79" s="70" t="s">
         <v>277</v>
       </c>
-      <c r="D79" s="65"/>
+      <c r="D79" s="70"/>
     </row>
     <row r="80" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C80" s="65"/>
-      <c r="D80" s="65"/>
+      <c r="C80" s="70"/>
+      <c r="D80" s="70"/>
     </row>
     <row r="81" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="82" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -5808,30 +5802,30 @@
       </c>
     </row>
     <row r="86" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C86" s="66" t="s">
+      <c r="C86" s="69" t="s">
         <v>283</v>
       </c>
-      <c r="D86" s="65"/>
-      <c r="E86" s="65"/>
-      <c r="F86" s="65"/>
+      <c r="D86" s="70"/>
+      <c r="E86" s="70"/>
+      <c r="F86" s="70"/>
     </row>
     <row r="87" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C87" s="65"/>
-      <c r="D87" s="65"/>
-      <c r="E87" s="65"/>
-      <c r="F87" s="65"/>
+      <c r="C87" s="70"/>
+      <c r="D87" s="70"/>
+      <c r="E87" s="70"/>
+      <c r="F87" s="70"/>
     </row>
     <row r="88" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C88" s="65"/>
-      <c r="D88" s="65"/>
-      <c r="E88" s="65"/>
-      <c r="F88" s="65"/>
+      <c r="C88" s="70"/>
+      <c r="D88" s="70"/>
+      <c r="E88" s="70"/>
+      <c r="F88" s="70"/>
     </row>
     <row r="89" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C89" s="65"/>
-      <c r="D89" s="65"/>
-      <c r="E89" s="65"/>
-      <c r="F89" s="65"/>
+      <c r="C89" s="70"/>
+      <c r="D89" s="70"/>
+      <c r="E89" s="70"/>
+      <c r="F89" s="70"/>
     </row>
     <row r="90" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="91" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5848,18 +5842,18 @@
       </c>
     </row>
     <row r="93" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="67" t="s">
+      <c r="B93" s="72" t="s">
         <v>280</v>
       </c>
-      <c r="C93" s="67"/>
+      <c r="C93" s="72"/>
     </row>
     <row r="94" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B94" s="65"/>
-      <c r="C94" s="65"/>
+      <c r="B94" s="70"/>
+      <c r="C94" s="70"/>
     </row>
     <row r="95" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B95" s="65"/>
-      <c r="C95" s="65"/>
+      <c r="B95" s="70"/>
+      <c r="C95" s="70"/>
     </row>
     <row r="96" spans="2:7" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="97" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -5882,11 +5876,11 @@
       </c>
     </row>
     <row r="99" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="68" t="s">
+      <c r="B99" s="71" t="s">
         <v>281</v>
       </c>
-      <c r="C99" s="68"/>
-      <c r="D99" s="68"/>
+      <c r="C99" s="71"/>
+      <c r="D99" s="71"/>
       <c r="F99" s="14" t="s">
         <v>112</v>
       </c>
@@ -5901,14 +5895,14 @@
       </c>
     </row>
     <row r="100" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="68"/>
-      <c r="C100" s="68"/>
-      <c r="D100" s="68"/>
+      <c r="B100" s="71"/>
+      <c r="C100" s="71"/>
+      <c r="D100" s="71"/>
     </row>
     <row r="101" spans="2:9" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B101" s="68"/>
-      <c r="C101" s="68"/>
-      <c r="D101" s="68"/>
+      <c r="B101" s="71"/>
+      <c r="C101" s="71"/>
+      <c r="D101" s="71"/>
       <c r="F101" s="31" t="s">
         <v>297</v>
       </c>
@@ -6808,7 +6802,7 @@
         <v>404</v>
       </c>
       <c r="M18" s="57" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="N18" s="17"/>
     </row>
@@ -7171,7 +7165,7 @@
     <row r="42" spans="8:14" ht="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="43" spans="8:14" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="J43" s="1" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="44" spans="8:14" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -7179,10 +7173,10 @@
         <v>1</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
     </row>
     <row r="45" spans="8:14" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -7193,7 +7187,7 @@
         <v>410</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
     </row>
     <row r="46" spans="8:14" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -7597,15 +7591,15 @@
       <c r="K16" s="24"/>
     </row>
     <row r="17" spans="2:11" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="G17" s="63"/>
-      <c r="H17" s="63"/>
-      <c r="I17" s="63"/>
+      <c r="C17" s="65"/>
+      <c r="D17" s="65"/>
+      <c r="E17" s="65"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="67"/>
+      <c r="I17" s="67"/>
     </row>
     <row r="18" spans="2:11" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="10" t="s">
@@ -7617,12 +7611,12 @@
       <c r="I18" s="19"/>
     </row>
     <row r="19" spans="2:11" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="62"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="62"/>
+      <c r="C19" s="66"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="66"/>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
     </row>
@@ -7634,12 +7628,12 @@
       <c r="K20" s="17"/>
     </row>
     <row r="21" spans="2:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="64"/>
-      <c r="D21" s="64"/>
-      <c r="E21" s="64"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="68"/>
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
@@ -7654,32 +7648,32 @@
       <c r="K22" s="20"/>
     </row>
     <row r="23" spans="2:11" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="65" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="61"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="61"/>
+      <c r="C23" s="65"/>
+      <c r="D23" s="65"/>
+      <c r="E23" s="65"/>
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
     </row>
     <row r="24" spans="2:11" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="61" t="s">
+      <c r="B24" s="65" t="s">
         <v>339</v>
       </c>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
     </row>
     <row r="25" spans="2:11" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="61" t="s">
+      <c r="B25" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-      <c r="E25" s="62"/>
+      <c r="C25" s="66"/>
+      <c r="D25" s="66"/>
+      <c r="E25" s="66"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
       <c r="H25" s="4"/>
@@ -7929,10 +7923,10 @@
     </row>
     <row r="4" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>64</v>
@@ -7944,34 +7938,34 @@
         <v>420</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
@@ -7981,10 +7975,10 @@
     </row>
     <row r="5" spans="2:21" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="38" t="s">
-        <v>427</v>
+        <v>489</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="D5" s="38" t="s">
         <v>70</v>
@@ -7996,34 +7990,34 @@
         <v>421</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="I5" s="38" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="L5" s="38" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="N5" s="38" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="O5" s="38" t="s">
         <v>85</v>
       </c>
       <c r="P5" s="38" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="Q5" s="8"/>
       <c r="R5" s="25"/>
@@ -8033,10 +8027,10 @@
     </row>
     <row r="6" spans="2:21" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
-        <v>428</v>
+        <v>490</v>
       </c>
       <c r="C6" s="58" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>72</v>
@@ -8048,34 +8042,34 @@
         <v>422</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="H6" s="70" t="s">
-        <v>449</v>
+        <v>436</v>
+      </c>
+      <c r="H6" s="62" t="s">
+        <v>446</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="Q6" s="3"/>
       <c r="R6" s="18"/>
@@ -8085,10 +8079,10 @@
     </row>
     <row r="7" spans="2:21" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
-        <v>429</v>
+        <v>491</v>
       </c>
       <c r="C7" s="58" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="D7" s="26" t="s">
         <v>91</v>
@@ -8098,28 +8092,28 @@
         <v>423</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
       <c r="O7" s="3" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="18"/>
@@ -8130,33 +8124,33 @@
     <row r="8" spans="2:21" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
       <c r="C8" s="3" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="59" t="s">
         <v>424</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>440</v>
-      </c>
-      <c r="H8" s="71"/>
+        <v>437</v>
+      </c>
+      <c r="H8" s="63"/>
       <c r="I8" s="3" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="J8" s="26" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
       <c r="O8" s="3" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="P8" s="5" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="18"/>
@@ -8167,7 +8161,7 @@
     <row r="9" spans="2:21" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3"/>
       <c r="C9" s="58" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="4"/>
@@ -8175,22 +8169,22 @@
         <v>425</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="H9" s="26"/>
       <c r="I9" s="3" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
       <c r="P9" s="3" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
@@ -8201,7 +8195,7 @@
     <row r="10" spans="2:21" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3"/>
       <c r="C10" s="36" t="s">
-        <v>71</v>
+        <v>542</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -8209,20 +8203,20 @@
         <v>426</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="Q10" s="18"/>
       <c r="R10" s="3"/>
@@ -8237,7 +8231,7 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="26" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -8248,7 +8242,7 @@
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="26" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
@@ -8342,18 +8336,18 @@
     </row>
     <row r="17" spans="3:18" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C17" s="3"/>
-      <c r="D17" s="61" t="s">
+      <c r="D17" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="63"/>
-      <c r="L17" s="63"/>
-      <c r="M17" s="63"/>
+      <c r="E17" s="65"/>
+      <c r="F17" s="65"/>
+      <c r="G17" s="65"/>
+      <c r="H17" s="65"/>
+      <c r="I17" s="65"/>
+      <c r="J17" s="65"/>
+      <c r="K17" s="67"/>
+      <c r="L17" s="67"/>
+      <c r="M17" s="67"/>
       <c r="O17" s="1">
         <v>1</v>
       </c>
@@ -8364,7 +8358,7 @@
         <v>0</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
     </row>
     <row r="18" spans="3:18" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -8385,15 +8379,15 @@
       </c>
     </row>
     <row r="19" spans="3:18" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="E19" s="62"/>
-      <c r="F19" s="62"/>
-      <c r="G19" s="62"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="62"/>
-      <c r="J19" s="62"/>
+      <c r="E19" s="66"/>
+      <c r="F19" s="66"/>
+      <c r="G19" s="66"/>
+      <c r="H19" s="66"/>
+      <c r="I19" s="66"/>
+      <c r="J19" s="66"/>
       <c r="N19" s="17"/>
       <c r="O19" s="17">
         <v>3</v>
@@ -8421,15 +8415,15 @@
       </c>
     </row>
     <row r="21" spans="3:18" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D21" s="61" t="s">
+      <c r="D21" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="64"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="64"/>
-      <c r="H21" s="64"/>
-      <c r="I21" s="64"/>
-      <c r="J21" s="64"/>
+      <c r="E21" s="68"/>
+      <c r="F21" s="68"/>
+      <c r="G21" s="68"/>
+      <c r="H21" s="68"/>
+      <c r="I21" s="68"/>
+      <c r="J21" s="68"/>
       <c r="N21" s="17"/>
       <c r="O21" s="1">
         <v>5</v>
@@ -8441,7 +8435,7 @@
         <v>1</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="22" spans="3:18" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -8463,15 +8457,15 @@
       </c>
     </row>
     <row r="23" spans="3:18" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="65" t="s">
         <v>50</v>
       </c>
-      <c r="E23" s="61"/>
-      <c r="F23" s="61"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="61"/>
+      <c r="E23" s="65"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="65"/>
+      <c r="H23" s="65"/>
+      <c r="I23" s="65"/>
+      <c r="J23" s="65"/>
       <c r="N23" s="7"/>
       <c r="O23" s="17">
         <v>7</v>
@@ -8484,15 +8478,15 @@
       </c>
     </row>
     <row r="24" spans="3:18" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D24" s="61" t="s">
+      <c r="D24" s="65" t="s">
         <v>339</v>
       </c>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="62"/>
-      <c r="H24" s="62"/>
-      <c r="I24" s="62"/>
-      <c r="J24" s="62"/>
+      <c r="E24" s="66"/>
+      <c r="F24" s="66"/>
+      <c r="G24" s="66"/>
+      <c r="H24" s="66"/>
+      <c r="I24" s="66"/>
+      <c r="J24" s="66"/>
       <c r="N24" s="7"/>
       <c r="O24" s="17">
         <v>8</v>
@@ -8505,15 +8499,15 @@
       </c>
     </row>
     <row r="25" spans="3:18" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D25" s="61" t="s">
+      <c r="D25" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="62"/>
-      <c r="F25" s="62"/>
-      <c r="G25" s="62"/>
-      <c r="H25" s="62"/>
-      <c r="I25" s="62"/>
-      <c r="J25" s="62"/>
+      <c r="E25" s="66"/>
+      <c r="F25" s="66"/>
+      <c r="G25" s="66"/>
+      <c r="H25" s="66"/>
+      <c r="I25" s="66"/>
+      <c r="J25" s="66"/>
       <c r="K25" s="15"/>
       <c r="L25" s="4"/>
       <c r="P25" s="15"/>
@@ -8740,18 +8734,18 @@
   <sheetData>
     <row r="2" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="38" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -8759,7 +8753,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="D4" s="3">
         <v>2</v>
@@ -8770,7 +8764,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="D5" s="3">
         <v>2</v>
@@ -8781,7 +8775,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D6" s="3">
         <v>2</v>
@@ -8792,7 +8786,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="D7" s="3">
         <v>2</v>
@@ -8803,7 +8797,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="D8" s="3">
         <v>2</v>
@@ -9120,27 +9114,27 @@
     </row>
     <row r="43" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="E43" s="43" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
     </row>
     <row r="44" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C44" s="58" t="s">
+        <v>430</v>
+      </c>
+      <c r="D44" s="58" t="s">
+        <v>431</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="C44" s="58" t="s">
+      <c r="F44" s="58" t="s">
         <v>433</v>
-      </c>
-      <c r="D44" s="58" t="s">
-        <v>434</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>435</v>
-      </c>
-      <c r="F44" s="58" t="s">
-        <v>436</v>
       </c>
       <c r="G44" s="36" t="s">
         <v>71</v>
@@ -9148,85 +9142,85 @@
     </row>
     <row r="45" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="C45" s="28" t="s">
+        <v>498</v>
+      </c>
+      <c r="D45" s="28">
+        <v>1</v>
+      </c>
+      <c r="E45" s="52" t="s">
         <v>500</v>
       </c>
-      <c r="C45" s="28" t="s">
+      <c r="F45" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="G45" s="28" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="61"/>
+      <c r="C46" s="28" t="s">
+        <v>504</v>
+      </c>
+      <c r="D46" s="28">
+        <v>2</v>
+      </c>
+      <c r="E46" s="28" t="s">
         <v>501</v>
       </c>
-      <c r="D45" s="28">
-        <v>1</v>
-      </c>
-      <c r="E45" s="52" t="s">
-        <v>503</v>
-      </c>
-      <c r="F45" s="28" t="s">
-        <v>508</v>
-      </c>
-      <c r="G45" s="28" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="46" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="69"/>
-      <c r="C46" s="28" t="s">
-        <v>507</v>
-      </c>
-      <c r="D46" s="28">
-        <v>2</v>
-      </c>
-      <c r="E46" s="28" t="s">
-        <v>504</v>
-      </c>
       <c r="F46" s="28" t="s">
+        <v>506</v>
+      </c>
+      <c r="G46" s="28" t="s">
         <v>509</v>
       </c>
-      <c r="G46" s="28" t="s">
-        <v>512</v>
-      </c>
     </row>
     <row r="47" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="69"/>
+      <c r="B47" s="61"/>
       <c r="C47" s="28" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="D47" s="28">
         <v>3</v>
       </c>
       <c r="E47" s="52"/>
       <c r="F47" s="28" t="s">
-        <v>510</v>
-      </c>
-      <c r="G47" s="69"/>
+        <v>507</v>
+      </c>
+      <c r="G47" s="61"/>
     </row>
     <row r="48" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="69"/>
+      <c r="B48" s="61"/>
       <c r="C48" s="28" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="D48" s="28">
         <v>4</v>
       </c>
       <c r="E48" s="52"/>
       <c r="F48" s="29" t="s">
-        <v>511</v>
-      </c>
-      <c r="G48" s="69"/>
+        <v>508</v>
+      </c>
+      <c r="G48" s="61"/>
     </row>
     <row r="49" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="69"/>
+      <c r="B49" s="61"/>
       <c r="C49" s="28" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="D49" s="28">
         <v>5</v>
       </c>
       <c r="E49" s="52"/>
-      <c r="F49" s="69"/>
-      <c r="G49" s="69"/>
+      <c r="F49" s="61"/>
+      <c r="G49" s="61"/>
     </row>
     <row r="51" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="2" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="C51" s="27"/>
       <c r="D51" s="27"/>
@@ -9237,13 +9231,13 @@
         <v>85</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
     </row>
     <row r="53" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9413,46 +9407,46 @@
     </row>
     <row r="66" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="27" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="67" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C67" s="66" t="s">
-        <v>516</v>
-      </c>
-      <c r="D67" s="65"/>
-      <c r="E67" s="65"/>
-      <c r="F67" s="65"/>
+      <c r="C67" s="69" t="s">
+        <v>513</v>
+      </c>
+      <c r="D67" s="70"/>
+      <c r="E67" s="70"/>
+      <c r="F67" s="70"/>
     </row>
     <row r="68" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C68" s="65"/>
-      <c r="D68" s="65"/>
-      <c r="E68" s="65"/>
-      <c r="F68" s="65"/>
+      <c r="C68" s="70"/>
+      <c r="D68" s="70"/>
+      <c r="E68" s="70"/>
+      <c r="F68" s="70"/>
     </row>
     <row r="69" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C69" s="65"/>
-      <c r="D69" s="65"/>
-      <c r="E69" s="65"/>
-      <c r="F69" s="65"/>
+      <c r="C69" s="70"/>
+      <c r="D69" s="70"/>
+      <c r="E69" s="70"/>
+      <c r="F69" s="70"/>
     </row>
     <row r="70" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C70" s="65"/>
-      <c r="D70" s="65"/>
-      <c r="E70" s="65"/>
-      <c r="F70" s="65"/>
+      <c r="C70" s="70"/>
+      <c r="D70" s="70"/>
+      <c r="E70" s="70"/>
+      <c r="F70" s="70"/>
     </row>
     <row r="72" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="2" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="73" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="38" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="74" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9460,7 +9454,7 @@
         <v>1</v>
       </c>
       <c r="C74" s="27" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="75" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9468,7 +9462,7 @@
         <v>2</v>
       </c>
       <c r="C75" s="27" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
     </row>
     <row r="76" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9476,7 +9470,7 @@
         <v>3</v>
       </c>
       <c r="C76" s="27" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="77" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9488,7 +9482,7 @@
         <v>81</v>
       </c>
       <c r="C79" s="27" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="D79" s="27"/>
       <c r="E79" s="27"/>
@@ -9521,7 +9515,7 @@
         <v>1</v>
       </c>
       <c r="C81" s="28" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="D81" s="29" t="s">
         <v>180</v>
@@ -9541,7 +9535,7 @@
         <v>2</v>
       </c>
       <c r="C82" s="28" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="D82" s="28" t="s">
         <v>181</v>
@@ -9561,7 +9555,7 @@
         <v>3</v>
       </c>
       <c r="C83" s="28" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="D83" s="28" t="s">
         <v>182</v>
@@ -9581,7 +9575,7 @@
         <v>4</v>
       </c>
       <c r="C84" s="28" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="D84" s="28" t="s">
         <v>183</v>
@@ -9601,7 +9595,7 @@
         <v>5</v>
       </c>
       <c r="C85" s="28" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="D85" s="28" t="s">
         <v>184</v>
@@ -9621,7 +9615,7 @@
         <v>6</v>
       </c>
       <c r="C86" s="28" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="D86" s="28" t="s">
         <v>185</v>
@@ -9641,7 +9635,7 @@
         <v>7</v>
       </c>
       <c r="C87" s="28" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="D87" s="28" t="s">
         <v>186</v>
@@ -9661,7 +9655,7 @@
         <v>8</v>
       </c>
       <c r="C88" s="28" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D88" s="28" t="s">
         <v>187</v>
@@ -9681,7 +9675,7 @@
         <v>9</v>
       </c>
       <c r="C89" s="28" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="D89" s="28" t="s">
         <v>188</v>
@@ -9701,7 +9695,7 @@
         <v>10</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="D90" s="28" t="s">
         <v>189</v>
@@ -9718,53 +9712,53 @@
     </row>
     <row r="92" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B92" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
     </row>
     <row r="93" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B93" s="38" t="s">
+        <v>435</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="D93" s="3" t="s">
         <v>438</v>
       </c>
-      <c r="C93" s="3" t="s">
-        <v>439</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>441</v>
-      </c>
       <c r="E93" s="3" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="F93" s="26" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="H93" s="26" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="94" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="28" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="D94" s="28">
         <v>258288995</v>
       </c>
       <c r="E94" s="28" t="s">
+        <v>530</v>
+      </c>
+      <c r="F94" s="28" t="s">
+        <v>532</v>
+      </c>
+      <c r="G94" s="28" t="s">
         <v>533</v>
       </c>
-      <c r="F94" s="28" t="s">
-        <v>535</v>
-      </c>
-      <c r="G94" s="28" t="s">
-        <v>536</v>
-      </c>
       <c r="H94" s="28" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
     </row>
     <row r="95" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9775,7 +9769,7 @@
       <c r="F95" s="28"/>
       <c r="G95" s="28"/>
       <c r="H95" s="28" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -9786,43 +9780,43 @@
       <c r="F96" s="28"/>
       <c r="G96" s="28"/>
       <c r="H96" s="28" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
     </row>
     <row r="98" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="2" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="C98" s="27"/>
       <c r="D98" s="27"/>
     </row>
     <row r="99" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="38" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="C99" s="38" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="100" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="68" t="s">
+      <c r="B100" s="71" t="s">
         <v>281</v>
       </c>
-      <c r="C100" s="68"/>
-      <c r="D100" s="68"/>
+      <c r="C100" s="71"/>
+      <c r="D100" s="71"/>
     </row>
     <row r="101" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B101" s="68"/>
-      <c r="C101" s="68"/>
-      <c r="D101" s="68"/>
+      <c r="B101" s="71"/>
+      <c r="C101" s="71"/>
+      <c r="D101" s="71"/>
     </row>
     <row r="102" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="68"/>
-      <c r="C102" s="68"/>
-      <c r="D102" s="68"/>
+      <c r="B102" s="71"/>
+      <c r="C102" s="71"/>
+      <c r="D102" s="71"/>
     </row>
     <row r="103" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B103" s="28">
@@ -10375,7 +10369,7 @@
       </c>
     </row>
     <row r="154" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B154" s="72" t="s">
+      <c r="B154" s="64" t="s">
         <v>111</v>
       </c>
       <c r="C154" s="27"/>
@@ -10390,7 +10384,7 @@
         <v>112</v>
       </c>
       <c r="D155" s="28" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="E155" s="4" t="s">
         <v>114</v>
@@ -10401,7 +10395,7 @@
     </row>
     <row r="156" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B156" s="27" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="C156" s="27"/>
       <c r="D156" s="27"/>
@@ -10467,22 +10461,22 @@
       <c r="F161" s="27"/>
     </row>
     <row r="163" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B163" s="72" t="s">
-        <v>468</v>
+      <c r="B163" s="64" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="164" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B164" s="38" t="s">
+        <v>466</v>
+      </c>
+      <c r="C164" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="D164" s="3" t="s">
+        <v>468</v>
+      </c>
+      <c r="E164" s="26" t="s">
         <v>469</v>
-      </c>
-      <c r="C164" s="3" t="s">
-        <v>470</v>
-      </c>
-      <c r="D164" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="E164" s="26" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="166" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
@@ -10591,7 +10585,7 @@
     </row>
     <row r="176" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B176" s="32" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="C176" s="27"/>
       <c r="D176" s="27"/>
@@ -10603,28 +10597,28 @@
     </row>
     <row r="177" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B177" s="14" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="C177" s="3" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="D177" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="E177" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="F177" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="G177" s="3" t="s">
         <v>540</v>
       </c>
-      <c r="E177" s="3" t="s">
+      <c r="H177" s="3" t="s">
         <v>541</v>
       </c>
-      <c r="F177" s="3" t="s">
-        <v>542</v>
-      </c>
-      <c r="G177" s="3" t="s">
-        <v>543</v>
-      </c>
-      <c r="H177" s="3" t="s">
-        <v>544</v>
-      </c>
       <c r="I177" s="4" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
     </row>
     <row r="178" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>